<commit_message>
fixat nästan hela denna grund next och påböjat denna avancerad standard
</commit_message>
<xml_diff>
--- a/docs/downloads/nextgen/Centrallager.xlsx
+++ b/docs/downloads/nextgen/Centrallager.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centrallager" sheetId="1" r:id="R46945e41221547bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centrallager" sheetId="1" r:id="R13a7c1efe9c24df7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -155,14 +155,14 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="8">
     <x:dxf>
       <x:font>
         <x:b/>
         <x:color rgb="FF173F35"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDE7E1"/>
         </x:patternFill>
       </x:fill>
@@ -173,7 +173,7 @@
         <x:color rgb="FF7A4A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4E4BF"/>
         </x:patternFill>
       </x:fill>
@@ -184,8 +184,59 @@
         <x:color rgb="FF8A2E20"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2D1CB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF36564B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5ECEA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FFB3261E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF36564B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE5ECEA"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB3261E"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -194,9 +245,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Centrallager" displayName="Centrallager" ref="A1:K26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:K26"/>
-  <x:tableColumns count="11">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Centrallager" displayName="Centrallager" ref="A1:L26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="Title"/>
     <x:tableColumn id="2" name="SKU"/>
     <x:tableColumn id="3" name="ProductModelID"/>
@@ -208,6 +258,7 @@
     <x:tableColumn id="9" name="IncomingQuantity"/>
     <x:tableColumn id="10" name="NextRestockDate"/>
     <x:tableColumn id="11" name="SalesStatus"/>
+    <x:tableColumn id="12" name="ReplenishmentCode"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -419,6 +470,7 @@
     <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -455,6 +507,9 @@
       <x:c r="K1" s="5" t="str">
         <x:v>SalesStatus</x:v>
       </x:c>
+      <x:c r="L1" t="str">
+        <x:v>ReplenishmentCode</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="10" t="str">
@@ -490,6 +545,9 @@
       <x:c r="K2" s="10" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L2" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="34" customHeight="1">
       <x:c r="A3" s="11" t="str">
@@ -525,6 +583,9 @@
       <x:c r="K3" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L3" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="11" t="str">
@@ -560,6 +621,9 @@
       <x:c r="K4" s="11" t="str">
         <x:v>Backorder</x:v>
       </x:c>
+      <x:c r="L4" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
       <x:c r="A5" s="11" t="str">
@@ -593,6 +657,9 @@
       <x:c r="K5" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L5" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="34" customHeight="1">
       <x:c r="A6" s="11" t="str">
@@ -628,6 +695,9 @@
       <x:c r="K6" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L6" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
       <x:c r="A7" s="11" t="str">
@@ -661,6 +731,9 @@
       <x:c r="K7" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L7" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
       <x:c r="A8" s="11" t="str">
@@ -696,6 +769,9 @@
       <x:c r="K8" s="11" t="str">
         <x:v>Backorder</x:v>
       </x:c>
+      <x:c r="L8" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
       <x:c r="A9" s="11" t="str">
@@ -731,6 +807,9 @@
       <x:c r="K9" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L9" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="34" customHeight="1">
       <x:c r="A10" s="11" t="str">
@@ -766,6 +845,9 @@
       <x:c r="K10" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L10" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="11" t="str">
@@ -799,6 +881,9 @@
       <x:c r="K11" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L11" t="str">
+        <x:v>RC90</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="11" t="str">
@@ -834,6 +919,9 @@
       <x:c r="K12" s="11" t="str">
         <x:v>Backorder</x:v>
       </x:c>
+      <x:c r="L12" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="11" t="str">
@@ -867,6 +955,9 @@
       <x:c r="K13" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L13" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="11" t="str">
@@ -902,6 +993,9 @@
       <x:c r="K14" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L14" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
       <x:c r="A15" s="11" t="str">
@@ -937,6 +1031,9 @@
       <x:c r="K15" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L15" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
       <x:c r="A16" s="11" t="str">
@@ -972,6 +1069,9 @@
       <x:c r="K16" s="11" t="str">
         <x:v>Backorder</x:v>
       </x:c>
+      <x:c r="L16" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="11" t="str">
@@ -1007,6 +1107,9 @@
       <x:c r="K17" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L17" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
       <x:c r="A18" s="11" t="str">
@@ -1040,6 +1143,9 @@
       <x:c r="K18" s="11" t="str">
         <x:v>Blocked</x:v>
       </x:c>
+      <x:c r="L18" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
       <x:c r="A19" s="11" t="str">
@@ -1073,6 +1179,9 @@
       <x:c r="K19" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L19" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="11" t="str">
@@ -1108,6 +1217,9 @@
       <x:c r="K20" s="11" t="str">
         <x:v>Backorder</x:v>
       </x:c>
+      <x:c r="L20" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
       <x:c r="A21" s="11" t="str">
@@ -1141,6 +1253,9 @@
       <x:c r="K21" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L21" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
       <x:c r="A22" s="11" t="str">
@@ -1176,6 +1291,9 @@
       <x:c r="K22" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L22" t="str">
+        <x:v>RC90</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="34" customHeight="1">
       <x:c r="A23" s="11" t="str">
@@ -1209,6 +1327,9 @@
       <x:c r="K23" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L23" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="34" customHeight="1">
       <x:c r="A24" s="11" t="str">
@@ -1244,6 +1365,9 @@
       <x:c r="K24" s="11" t="str">
         <x:v>Backorder</x:v>
       </x:c>
+      <x:c r="L24" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="34" customHeight="1">
       <x:c r="A25" s="11" t="str">
@@ -1279,6 +1403,9 @@
       <x:c r="K25" s="11" t="str">
         <x:v>Available</x:v>
       </x:c>
+      <x:c r="L25" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="34" customHeight="1">
       <x:c r="A26" s="12" t="str">
@@ -1312,21 +1439,31 @@
       <x:c r="K26" s="12" t="str">
         <x:v>Blocked</x:v>
       </x:c>
+      <x:c r="L26" t="str">
+        <x:v>RC10</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="K2:K26">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Available"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Backorder"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Blocked"/>
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Available"/>
+    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Backorder"/>
+    <x:cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="Blocked"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="L2:L26">
+    <x:cfRule type="containsText" dxfId="6" priority="4" operator="containsText" text="RC10"/>
+    <x:cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="RC90"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="K2:K26">
       <x:formula1>"Available,Backorder,Blocked"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L2:L26">
+      <x:formula1>"RC10,RC90"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc725311a6da448bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0295fcc39df4f55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>